<commit_message>
Automatic update of files.
</commit_message>
<xml_diff>
--- a/Översikt OKÄNT.xlsx
+++ b/Översikt OKÄNT.xlsx
@@ -569,7 +569,7 @@
         <v>43419</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -626,7 +626,7 @@
         <v>43690</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -683,7 +683,7 @@
         <v>43735</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -740,7 +740,7 @@
         <v>43780</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -797,7 +797,7 @@
         <v>43845</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -854,7 +854,7 @@
         <v>43864</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
         <v>43872</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -968,7 +968,7 @@
         <v>43971</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1025,7 +1025,7 @@
         <v>44005</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1082,7 +1082,7 @@
         <v>44098</v>
       </c>
       <c r="C11" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
         <v>44178</v>
       </c>
       <c r="C12" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1196,7 +1196,7 @@
         <v>44224</v>
       </c>
       <c r="C13" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1253,7 +1253,7 @@
         <v>44327</v>
       </c>
       <c r="C14" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1310,7 +1310,7 @@
         <v>44501</v>
       </c>
       <c r="C15" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1367,7 +1367,7 @@
         <v>44707</v>
       </c>
       <c r="C16" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1424,7 +1424,7 @@
         <v>44729</v>
       </c>
       <c r="C17" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1481,7 +1481,7 @@
         <v>44844</v>
       </c>
       <c r="C18" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1538,7 +1538,7 @@
         <v>45040</v>
       </c>
       <c r="C19" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1595,7 +1595,7 @@
         <v>45086</v>
       </c>
       <c r="C20" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1652,7 +1652,7 @@
         <v>45092</v>
       </c>
       <c r="C21" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1709,7 +1709,7 @@
         <v>45092</v>
       </c>
       <c r="C22" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1766,7 +1766,7 @@
         <v>45121</v>
       </c>
       <c r="C23" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
         <v>45124</v>
       </c>
       <c r="C24" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1880,7 +1880,7 @@
         <v>45154</v>
       </c>
       <c r="C25" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1937,7 +1937,7 @@
         <v>45154</v>
       </c>
       <c r="C26" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1994,7 +1994,7 @@
         <v>45253</v>
       </c>
       <c r="C27" s="1" t="n">
-        <v>45337</v>
+        <v>45338</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>

</xml_diff>